<commit_message>
Updated POL_grids_kan model - 2026-06-30 01:14
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_POL_grids_kan/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AFBA5AA-491D-459E-AF22-30A7CA7DFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E29EFB6-6A66-4CC3-AD7E-EE114402D970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -853,18 +853,54 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_POL_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_006</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_013</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_010</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_011</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 11</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_POL_001</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 1</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_POL_002</t>
   </si>
   <si>
@@ -877,6 +913,60 @@
     <t>connecting solar to buses in cluster 20</t>
   </si>
   <si>
+    <t>distr_solelc_spv_POL_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_018</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_016</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_017</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 17</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_007</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_POL_012</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 12</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_POL_015</t>
   </si>
   <si>
@@ -889,102 +979,30 @@
     <t>connecting solar to buses in cluster 19</t>
   </si>
   <si>
-    <t>distr_solelc_spv_POL_010</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_006</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_013</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 13</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_017</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 17</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_018</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 18</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_016</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_007</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_012</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_POL_011</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 11</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_w255293400-220_POL,e_w46235456-400_POL,e_w385118244-400_POL,e_w46092396-400_POL,e_PL3-220_POL,e_w112614319-400_POL,e_PL6-220_POL</t>
+  </si>
+  <si>
+    <t>e_w144646702-400_POL,e_w101914781-220_POL,e_w101914781-400_POL,e_PL24-220_POL,e_w101915790-220_POL</t>
+  </si>
+  <si>
+    <t>e_w726776987-220_POL,e_w170368942-220_POL,e_w148060965-400_POL,e_w173613665-220_POL,e_w194903381-400_POL</t>
+  </si>
+  <si>
+    <t>e_w303870256-400_POL,e_w170259740-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255972397-400_POL,e_PL27-400_POL,e_PL17-400_POL,e_w194903381-400_POL,e_w293489663-400_POL</t>
+  </si>
+  <si>
+    <t>e_w121656686-220_POL,e_w121656686-400_POL,e_w255972326-400_POL,e_w303870256-400_POL,e_PL17-400_POL,e_w293489663-400_POL,e_w170259740-220_POL</t>
+  </si>
+  <si>
     <t>e_PL40-220_POL,e_w158232924-220_POL,e_w178756295-220_POL,e_w111615226-400_POL,e_PL30-220_POL</t>
   </si>
   <si>
@@ -994,55 +1012,55 @@
     <t>e_w254235846-400_POL,e_w173582810-400_POL,e_w255973806-220_POL,e_w88544449-220_POL,e_w255972397-400_POL</t>
   </si>
   <si>
+    <t>e_w98634956-220_POL,e_w98611253-220_POL,e_w135598292-220_POL,e_w66051759-220_POL,e_w115801644-220_POL,e_w87667718-220_POL,e_w166710856-400_POL,e_PL61-220_POL</t>
+  </si>
+  <si>
+    <t>e_w145037309-220_POL,e_w29115701-220_POL,e_w91384044-400_POL,e_PL20-220_POL</t>
+  </si>
+  <si>
+    <t>e_w255293403-400_POL,e_w255284259-220_POL,e_w171383831-220_POL,e_w35366436-220_POL,e_PL21-220_POL</t>
+  </si>
+  <si>
+    <t>e_w180535363-220_POL,e_w32036484-220_POL,e_w238640596-220_POL,e_w175406958-220_POL,e_w32036484-400_POL,e_w238640596-400_POL,e_w254938713-400_POL,e_w255293400-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL18-400_POL,e_PL10-400_POL,e_PL4-220_POL,e_w668348943-220_POL,e_w385539724-220_POL,e_PL8-220_POL</t>
+  </si>
+  <si>
+    <t>e_w180542657-220_POL,e_w180535363-220_POL,e_PL46-220_POL,e_w154510504-400_POL,e_w148197330-220_POL,e_PL36-400_POL,e_w79033485-400_POL,e_w255293403-400_POL</t>
+  </si>
+  <si>
+    <t>e_PL22-220_POL,e_PL15-400_POL,e_w72879943-220_POL,e_w143484238-220_POL,e_w658600169-400_POL,e_w144646702-400_POL</t>
+  </si>
+  <si>
+    <t>e_w175406958-220_POL,e_w175406958-400_POL,e_w178838661-220_POL,e_w255314292_POL,e_w534238983-400_POL,e_r18085709-400_POL</t>
+  </si>
+  <si>
+    <t>e_w166838338-400_POL,e_w191352746-220_POL,e_PL62-400_POL,e_w198635989-220_POL,e_w170368942-220_POL</t>
+  </si>
+  <si>
     <t>e_w185459155-220_POL,e_w336990960-220_POL,e_PL36-400_POL,e_w184899160-220_POL,e_w293489607-400_POL,e_PL41-400_POL,e_w171917072-400_POL,e_w241842600-400_POL,e_PL35-220_POL,e_w199098050-220_POL</t>
   </si>
   <si>
     <t>e_w199098050-220_POL,e_w145037309-220_POL,e_w228154083-220_POL,e_w189851841-220_POL,e_PL32-220_POL</t>
   </si>
   <si>
-    <t>e_w303870256-400_POL,e_w170259740-220_POL</t>
-  </si>
-  <si>
-    <t>e_w144646702-400_POL,e_w101914781-220_POL,e_w101914781-400_POL,e_PL24-220_POL,e_w101915790-220_POL</t>
-  </si>
-  <si>
-    <t>e_w726776987-220_POL,e_w170368942-220_POL,e_w148060965-400_POL,e_w173613665-220_POL,e_w194903381-400_POL</t>
-  </si>
-  <si>
-    <t>e_w180535363-220_POL,e_w32036484-220_POL,e_w238640596-220_POL,e_w175406958-220_POL,e_w32036484-400_POL,e_w238640596-400_POL,e_w254938713-400_POL,e_w255293400-220_POL</t>
-  </si>
-  <si>
-    <t>e_PL18-400_POL,e_PL10-400_POL,e_PL4-220_POL,e_w668348943-220_POL,e_w385539724-220_POL,e_PL8-220_POL</t>
-  </si>
-  <si>
-    <t>e_w180542657-220_POL,e_w180535363-220_POL,e_PL46-220_POL,e_w154510504-400_POL,e_w148197330-220_POL,e_PL36-400_POL,e_w79033485-400_POL,e_w255293403-400_POL</t>
-  </si>
-  <si>
-    <t>e_PL22-220_POL,e_PL15-400_POL,e_w72879943-220_POL,e_w143484238-220_POL,e_w658600169-400_POL,e_w144646702-400_POL</t>
-  </si>
-  <si>
-    <t>e_w98634956-220_POL,e_w98611253-220_POL,e_w135598292-220_POL,e_w66051759-220_POL,e_w115801644-220_POL,e_w87667718-220_POL,e_w166710856-400_POL,e_PL61-220_POL</t>
-  </si>
-  <si>
-    <t>e_w145037309-220_POL,e_w29115701-220_POL,e_w91384044-400_POL,e_PL20-220_POL</t>
-  </si>
-  <si>
-    <t>e_w255293403-400_POL,e_w255284259-220_POL,e_w171383831-220_POL,e_w35366436-220_POL,e_PL21-220_POL</t>
-  </si>
-  <si>
-    <t>e_w255972397-400_POL,e_PL27-400_POL,e_PL17-400_POL,e_w194903381-400_POL,e_w293489663-400_POL</t>
-  </si>
-  <si>
-    <t>e_w255293400-220_POL,e_w46235456-400_POL,e_w385118244-400_POL,e_w46092396-400_POL,e_PL3-220_POL,e_w112614319-400_POL,e_PL6-220_POL</t>
-  </si>
-  <si>
-    <t>e_w175406958-220_POL,e_w175406958-400_POL,e_w178838661-220_POL,e_w255314292_POL,e_w534238983-400_POL,e_r18085709-400_POL</t>
-  </si>
-  <si>
-    <t>e_w166838338-400_POL,e_w191352746-220_POL,e_PL62-400_POL,e_w198635989-220_POL,e_w170368942-220_POL</t>
-  </si>
-  <si>
-    <t>e_w121656686-220_POL,e_w121656686-400_POL,e_w255972326-400_POL,e_w303870256-400_POL,e_PL17-400_POL,e_w293489663-400_POL,e_w170259740-220_POL</t>
+    <t>distr_wonelc_won_POL_015</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 15</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_016</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 16</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_017</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 17</t>
   </si>
   <si>
     <t>distr_wonelc_won_POL_019</t>
@@ -1051,6 +1069,36 @@
     <t>connecting wind onshore to buses in cluster 19</t>
   </si>
   <si>
+    <t>distr_wonelc_won_POL_012</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 12</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_018</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 18</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_002</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_005</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 5</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_POL_009</t>
   </si>
   <si>
@@ -1063,6 +1111,24 @@
     <t>connecting wind onshore to buses in cluster 4</t>
   </si>
   <si>
+    <t>distr_wonelc_won_POL_007</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_POL_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_POL_013</t>
   </si>
   <si>
@@ -1075,24 +1141,6 @@
     <t>connecting wind onshore to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_007</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_POL_014</t>
   </si>
   <si>
@@ -1105,36 +1153,6 @@
     <t>connecting wind onshore to buses in cluster 20</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_015</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 15</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_016</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 16</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_002</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_005</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_017</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 17</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_POL_011</t>
   </si>
   <si>
@@ -1147,22 +1165,22 @@
     <t>connecting wind onshore to buses in cluster 10</t>
   </si>
   <si>
-    <t>distr_wonelc_won_POL_012</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 12</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_POL_018</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 18</t>
+    <t>elc_won_POL_015</t>
+  </si>
+  <si>
+    <t>e_w98634956-220_POL,e_w98611253-220_POL,e_w115801644-220_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_016</t>
+  </si>
+  <si>
+    <t>e_PL62-400_POL,e_w198635989-220_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_017</t>
+  </si>
+  <si>
+    <t>e_w166710856-400_POL,e_w166838338-400_POL</t>
   </si>
   <si>
     <t>elc_won_POL_019</t>
@@ -1171,6 +1189,36 @@
     <t>e_w135598292-220_POL,e_w66051759-220_POL,e_w241842600-400_POL,e_w115801644-220_POL,e_w87667718-220_POL,e_w199098050-220_POL</t>
   </si>
   <si>
+    <t>elc_won_POL_012</t>
+  </si>
+  <si>
+    <t>e_w158232924-220_POL,e_PL18-400_POL,e_PL10-400_POL,e_PL30-220_POL,e_w385539724-220_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_003</t>
+  </si>
+  <si>
+    <t>e_w255973806-220_POL,e_PL20-220_POL,e_w88544449-220_POL,e_w255972397-400_POL,e_w148060965-400_POL,e_PL27-400_POL,e_PL17-400_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_018</t>
+  </si>
+  <si>
+    <t>e_w178756295-220_POL,e_w177749653-220_POL,e_w179279860-220_POL,e_PL46-220_POL,e_w336990960-220_POL,e_w255277953-400_POL,e_PL36-400_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_002</t>
+  </si>
+  <si>
+    <t>e_PL61-220_POL,e_w228154083-220_POL,e_w189851841-220_POL,e_w191352746-220_POL,e_w254235846-400_POL,e_w173582810-400_POL,e_w726776987-220_POL,e_w88544449-220_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_005</t>
+  </si>
+  <si>
+    <t>e_w121656686-220_POL,e_w121656686-400_POL,e_w255972326-400_POL,e_w303870256-400_POL,e_w170259740-220_POL,e_PL17-400_POL,e_w293489663-400_POL,e_w194903381-400_POL</t>
+  </si>
+  <si>
     <t>elc_won_POL_009</t>
   </si>
   <si>
@@ -1180,6 +1228,24 @@
     <t>elc_won_POL_004</t>
   </si>
   <si>
+    <t>elc_won_POL_007</t>
+  </si>
+  <si>
+    <t>e_w145037309-220_POL,e_w144646702-400_POL,e_w101914781-220_POL,e_w91384044-400_POL,e_PL24-220_POL,e_w101915790-220_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_006</t>
+  </si>
+  <si>
+    <t>e_w255293403-400_POL,e_w255284259-220_POL,e_PL22-220_POL,e_PL15-400_POL,e_w171383831-220_POL,e_w72879943-220_POL,e_w143484238-220_POL,e_PL21-220_POL,e_w658600169-400_POL,e_w144646702-400_POL</t>
+  </si>
+  <si>
+    <t>elc_won_POL_001</t>
+  </si>
+  <si>
+    <t>e_PL35-220_POL,e_w35366436-220_POL,e_w199098050-220_POL,e_w145037309-220_POL,e_PL32-220_POL,e_w29115701-220_POL</t>
+  </si>
+  <si>
     <t>elc_won_POL_013</t>
   </si>
   <si>
@@ -1192,24 +1258,6 @@
     <t>e_w101914781-220_POL,e_w101914781-400_POL,e_w101915790-220_POL,e_w303870256-400_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_007</t>
-  </si>
-  <si>
-    <t>e_w145037309-220_POL,e_w144646702-400_POL,e_w101914781-220_POL,e_w91384044-400_POL,e_PL24-220_POL,e_w101915790-220_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_006</t>
-  </si>
-  <si>
-    <t>e_w255293403-400_POL,e_w255284259-220_POL,e_PL22-220_POL,e_PL15-400_POL,e_w171383831-220_POL,e_w72879943-220_POL,e_w143484238-220_POL,e_PL21-220_POL,e_w658600169-400_POL,e_w144646702-400_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_001</t>
-  </si>
-  <si>
-    <t>e_PL35-220_POL,e_w35366436-220_POL,e_w199098050-220_POL,e_w145037309-220_POL,e_PL32-220_POL,e_w29115701-220_POL</t>
-  </si>
-  <si>
     <t>elc_won_POL_014</t>
   </si>
   <si>
@@ -1222,36 +1270,6 @@
     <t>e_w185459155-220_POL,e_w336990960-220_POL,e_PL36-400_POL,e_w184899160-220_POL,e_w293489607-400_POL,e_PL41-400_POL,e_w171917072-400_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_015</t>
-  </si>
-  <si>
-    <t>e_w98634956-220_POL,e_w98611253-220_POL,e_w115801644-220_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_016</t>
-  </si>
-  <si>
-    <t>e_PL62-400_POL,e_w198635989-220_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_002</t>
-  </si>
-  <si>
-    <t>e_PL61-220_POL,e_w228154083-220_POL,e_w189851841-220_POL,e_w191352746-220_POL,e_w254235846-400_POL,e_w173582810-400_POL,e_w726776987-220_POL,e_w88544449-220_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_005</t>
-  </si>
-  <si>
-    <t>e_w121656686-220_POL,e_w121656686-400_POL,e_w255972326-400_POL,e_w303870256-400_POL,e_w170259740-220_POL,e_PL17-400_POL,e_w293489663-400_POL,e_w194903381-400_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_017</t>
-  </si>
-  <si>
-    <t>e_w166710856-400_POL,e_w166838338-400_POL</t>
-  </si>
-  <si>
     <t>elc_won_POL_011</t>
   </si>
   <si>
@@ -1264,22 +1282,16 @@
     <t>e_PL4-220_POL,e_w668348943-220_POL,e_PL8-220_POL,e_w175406958-220_POL,e_w175406958-400_POL,e_w238640596-400_POL,e_w178838661-220_POL,e_w255314292_POL,e_w255293400-220_POL,e_w534238983-400_POL,e_r18085709-400_POL,e_w46235456-400_POL,e_w385118244-400_POL</t>
   </si>
   <si>
-    <t>elc_won_POL_012</t>
-  </si>
-  <si>
-    <t>e_w158232924-220_POL,e_PL18-400_POL,e_PL10-400_POL,e_PL30-220_POL,e_w385539724-220_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_003</t>
-  </si>
-  <si>
-    <t>e_w255973806-220_POL,e_PL20-220_POL,e_w88544449-220_POL,e_w255972397-400_POL,e_w148060965-400_POL,e_PL27-400_POL,e_PL17-400_POL</t>
-  </si>
-  <si>
-    <t>elc_won_POL_018</t>
-  </si>
-  <si>
-    <t>e_w178756295-220_POL,e_w177749653-220_POL,e_w179279860-220_POL,e_PL46-220_POL,e_w336990960-220_POL,e_w255277953-400_POL,e_PL36-400_POL</t>
+    <t>distr_wofelc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 5</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
   </si>
   <si>
     <t>distr_wofelc_wof_POL_007</t>
@@ -1288,6 +1300,30 @@
     <t>connecting wind offshore to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_wofelc_wof_POL_008</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_003</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 6</t>
+  </si>
+  <si>
     <t>distr_wofelc_wof_POL_010</t>
   </si>
   <si>
@@ -1300,54 +1336,51 @@
     <t>connecting wind offshore to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_008</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_POL_003</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 3</t>
-  </si>
-  <si>
     <t>distr_wofelc_wof_POL_009</t>
   </si>
   <si>
     <t>connecting wind offshore to buses in cluster 9</t>
   </si>
   <si>
+    <t>elc_wof_POL_005</t>
+  </si>
+  <si>
+    <t>e_PL1-400_POL,e_w86494356-400_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_001</t>
+  </si>
+  <si>
+    <t>e_w112614319-400_POL</t>
+  </si>
+  <si>
     <t>elc_wof_POL_007</t>
   </si>
   <si>
     <t>e_w175406958-220_POL,e_w175406958-400_POL</t>
   </si>
   <si>
+    <t>elc_wof_POL_008</t>
+  </si>
+  <si>
+    <t>e_w668348943-220_POL,e_w175406958-220_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_003</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_004</t>
+  </si>
+  <si>
+    <t>e_w255314292_POL,e_PL1-400_POL</t>
+  </si>
+  <si>
+    <t>elc_wof_POL_006</t>
+  </si>
+  <si>
+    <t>e_PL1-400_POL</t>
+  </si>
+  <si>
     <t>elc_wof_POL_010</t>
   </si>
   <si>
@@ -1358,39 +1391,6 @@
   </si>
   <si>
     <t>e_w86494356-400_POL,e_w112614319-400_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_004</t>
-  </si>
-  <si>
-    <t>e_w255314292_POL,e_PL1-400_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_006</t>
-  </si>
-  <si>
-    <t>e_PL1-400_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_005</t>
-  </si>
-  <si>
-    <t>e_PL1-400_POL,e_w86494356-400_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_001</t>
-  </si>
-  <si>
-    <t>e_w112614319-400_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_008</t>
-  </si>
-  <si>
-    <t>e_w668348943-220_POL,e_w175406958-220_POL</t>
-  </si>
-  <si>
-    <t>elc_wof_POL_003</t>
   </si>
   <si>
     <t>elc_wof_POL_009</t>
@@ -7160,7 +7160,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD221FBF-3B29-4FC3-A0D0-F0125757B567}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F313D39-7B5E-4944-960D-E171BA1E2090}">
   <dimension ref="B9:BD30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7398,16 +7398,16 @@
         <v>241</v>
       </c>
       <c r="Y11" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="Z11" t="s">
         <v>285</v>
       </c>
       <c r="AA11">
-        <v>0.99733507264559695</v>
+        <v>0.99738245649758195</v>
       </c>
       <c r="AB11">
-        <v>48.857001497390002</v>
+        <v>47.988297544331637</v>
       </c>
       <c r="AD11" t="s">
         <v>240</v>
@@ -7440,10 +7440,10 @@
         <v>346</v>
       </c>
       <c r="AO11">
-        <v>0.99873239758997023</v>
+        <v>0.99641308487583879</v>
       </c>
       <c r="AP11">
-        <v>23.239377517213022</v>
+        <v>65.760110609622657</v>
       </c>
       <c r="AR11" t="s">
         <v>240</v>
@@ -7476,10 +7476,10 @@
         <v>405</v>
       </c>
       <c r="BC11">
-        <v>0.99603343715055259</v>
+        <v>0.9932866968373224</v>
       </c>
       <c r="BD11">
-        <v>72.720318906536249</v>
+        <v>123.07722464908932</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -7544,16 +7544,16 @@
         <v>245</v>
       </c>
       <c r="Y12" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="Z12" t="s">
         <v>286</v>
       </c>
       <c r="AA12">
-        <v>0.99583365539385327</v>
+        <v>0.99648087644372252</v>
       </c>
       <c r="AB12">
-        <v>76.382984446022675</v>
+        <v>64.517265198419722</v>
       </c>
       <c r="AD12" t="s">
         <v>240</v>
@@ -7586,10 +7586,10 @@
         <v>348</v>
       </c>
       <c r="AO12">
-        <v>0.99635146162488653</v>
+        <v>0.99449756685866841</v>
       </c>
       <c r="AP12">
-        <v>66.889870210414614</v>
+        <v>100.87794092441324</v>
       </c>
       <c r="AR12" t="s">
         <v>240</v>
@@ -7622,10 +7622,10 @@
         <v>407</v>
       </c>
       <c r="BC12">
-        <v>0.99609037037675463</v>
+        <v>0.99644388872049838</v>
       </c>
       <c r="BD12">
-        <v>71.676543092831025</v>
+        <v>65.195373457529499</v>
       </c>
     </row>
     <row r="13" spans="2:56">
@@ -7690,16 +7690,16 @@
         <v>247</v>
       </c>
       <c r="Y13" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="Z13" t="s">
         <v>287</v>
       </c>
       <c r="AA13">
-        <v>0.99875154162789404</v>
+        <v>0.99621535905375425</v>
       </c>
       <c r="AB13">
-        <v>22.888403488609324</v>
+        <v>69.385084014505708</v>
       </c>
       <c r="AD13" t="s">
         <v>240</v>
@@ -7729,13 +7729,13 @@
         <v>349</v>
       </c>
       <c r="AN13" t="s">
-        <v>292</v>
+        <v>350</v>
       </c>
       <c r="AO13">
-        <v>0.99586212495478665</v>
+        <v>0.99776911581804295</v>
       </c>
       <c r="AP13">
-        <v>75.861042495577635</v>
+        <v>40.899543335879912</v>
       </c>
       <c r="AR13" t="s">
         <v>240</v>
@@ -7768,10 +7768,10 @@
         <v>409</v>
       </c>
       <c r="BC13">
-        <v>0.99353710926584593</v>
+        <v>0.99603343715055259</v>
       </c>
       <c r="BD13">
-        <v>118.48633012615811</v>
+        <v>72.720318906536249</v>
       </c>
     </row>
     <row r="14" spans="2:56">
@@ -7836,16 +7836,16 @@
         <v>249</v>
       </c>
       <c r="Y14" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="Z14" t="s">
         <v>288</v>
       </c>
       <c r="AA14">
-        <v>0.99860106452186825</v>
+        <v>0.99511607748745434</v>
       </c>
       <c r="AB14">
-        <v>25.647150432415483</v>
+        <v>89.538579396670116</v>
       </c>
       <c r="AD14" t="s">
         <v>240</v>
@@ -7872,16 +7872,16 @@
         <v>311</v>
       </c>
       <c r="AM14" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AN14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="AO14">
-        <v>0.99883902037019667</v>
+        <v>0.99873239758997023</v>
       </c>
       <c r="AP14">
-        <v>21.284626546395259</v>
+        <v>23.239377517213022</v>
       </c>
       <c r="AR14" t="s">
         <v>240</v>
@@ -7914,10 +7914,10 @@
         <v>411</v>
       </c>
       <c r="BC14">
-        <v>0.99255696761939116</v>
+        <v>0.99383395234396599</v>
       </c>
       <c r="BD14">
-        <v>136.4555936444961</v>
+        <v>113.04420702728957</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -7982,16 +7982,16 @@
         <v>251</v>
       </c>
       <c r="Y15" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="Z15" t="s">
         <v>289</v>
       </c>
       <c r="AA15">
-        <v>0.99775856069920277</v>
+        <v>0.99572127940552169</v>
       </c>
       <c r="AB15">
-        <v>41.093053847949164</v>
+        <v>78.443210898768598</v>
       </c>
       <c r="AD15" t="s">
         <v>240</v>
@@ -8018,16 +8018,16 @@
         <v>313</v>
       </c>
       <c r="AM15" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN15" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AO15">
-        <v>0.99521984547821263</v>
+        <v>0.99749126227646956</v>
       </c>
       <c r="AP15">
-        <v>87.636166232768815</v>
+        <v>45.993524931390482</v>
       </c>
       <c r="AR15" t="s">
         <v>240</v>
@@ -8057,13 +8057,13 @@
         <v>412</v>
       </c>
       <c r="BB15" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="BC15">
-        <v>0.99615776238359954</v>
+        <v>0.99564789206089888</v>
       </c>
       <c r="BD15">
-        <v>70.441022967342263</v>
+        <v>79.788645550187297</v>
       </c>
     </row>
     <row r="16" spans="2:56">
@@ -8128,16 +8128,16 @@
         <v>253</v>
       </c>
       <c r="Y16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Z16" t="s">
         <v>290</v>
       </c>
       <c r="AA16">
-        <v>0.99511607748745434</v>
+        <v>0.99692898913090644</v>
       </c>
       <c r="AB16">
-        <v>89.538579396670116</v>
+        <v>56.301865933381954</v>
       </c>
       <c r="AD16" t="s">
         <v>240</v>
@@ -8164,16 +8164,16 @@
         <v>315</v>
       </c>
       <c r="AM16" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AN16" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="AO16">
-        <v>0.99653588726932718</v>
+        <v>0.99807543246352515</v>
       </c>
       <c r="AP16">
-        <v>63.508733395668145</v>
+        <v>35.283738168705199</v>
       </c>
       <c r="AR16" t="s">
         <v>240</v>
@@ -8200,16 +8200,16 @@
         <v>394</v>
       </c>
       <c r="BA16" t="s">
+        <v>413</v>
+      </c>
+      <c r="BB16" t="s">
         <v>414</v>
       </c>
-      <c r="BB16" t="s">
-        <v>415</v>
-      </c>
       <c r="BC16">
-        <v>0.9932866968373224</v>
+        <v>0.99255696761939116</v>
       </c>
       <c r="BD16">
-        <v>123.07722464908932</v>
+        <v>136.4555936444961</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -8274,16 +8274,16 @@
         <v>255</v>
       </c>
       <c r="Y17" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="Z17" t="s">
         <v>291</v>
       </c>
       <c r="AA17">
-        <v>0.99648087644372252</v>
+        <v>0.99733507264559695</v>
       </c>
       <c r="AB17">
-        <v>64.517265198419722</v>
+        <v>48.857001497390002</v>
       </c>
       <c r="AD17" t="s">
         <v>240</v>
@@ -8310,16 +8310,16 @@
         <v>317</v>
       </c>
       <c r="AM17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AN17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AO17">
-        <v>0.99826576737141715</v>
+        <v>0.99622969699231045</v>
       </c>
       <c r="AP17">
-        <v>31.794264857351436</v>
+        <v>69.122221807641537</v>
       </c>
       <c r="AR17" t="s">
         <v>240</v>
@@ -8346,16 +8346,16 @@
         <v>396</v>
       </c>
       <c r="BA17" t="s">
+        <v>415</v>
+      </c>
+      <c r="BB17" t="s">
         <v>416</v>
       </c>
-      <c r="BB17" t="s">
-        <v>417</v>
-      </c>
       <c r="BC17">
-        <v>0.99644388872049838</v>
+        <v>0.99615776238359954</v>
       </c>
       <c r="BD17">
-        <v>65.195373457529499</v>
+        <v>70.441022967342263</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -8420,16 +8420,16 @@
         <v>257</v>
       </c>
       <c r="Y18" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="Z18" t="s">
         <v>292</v>
       </c>
       <c r="AA18">
-        <v>0.99621535905375425</v>
+        <v>0.99583365539385327</v>
       </c>
       <c r="AB18">
-        <v>69.385084014505708</v>
+        <v>76.382984446022675</v>
       </c>
       <c r="AD18" t="s">
         <v>240</v>
@@ -8456,16 +8456,16 @@
         <v>319</v>
       </c>
       <c r="AM18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AN18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AO18">
-        <v>0.99871360797890252</v>
+        <v>0.99845079995590791</v>
       </c>
       <c r="AP18">
-        <v>23.583853720120768</v>
+        <v>28.402000808355538</v>
       </c>
       <c r="AR18" t="s">
         <v>240</v>
@@ -8492,16 +8492,16 @@
         <v>398</v>
       </c>
       <c r="BA18" t="s">
+        <v>417</v>
+      </c>
+      <c r="BB18" t="s">
         <v>418</v>
       </c>
-      <c r="BB18" t="s">
-        <v>419</v>
-      </c>
       <c r="BC18">
-        <v>0.99383395234396599</v>
+        <v>0.99609037037675463</v>
       </c>
       <c r="BD18">
-        <v>113.04420702728957</v>
+        <v>71.676543092831025</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -8566,16 +8566,16 @@
         <v>259</v>
       </c>
       <c r="Y19" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="Z19" t="s">
         <v>293</v>
       </c>
       <c r="AA19">
-        <v>0.99729953359766199</v>
+        <v>0.99875154162789404</v>
       </c>
       <c r="AB19">
-        <v>49.508550709529651</v>
+        <v>22.888403488609324</v>
       </c>
       <c r="AD19" t="s">
         <v>240</v>
@@ -8602,16 +8602,16 @@
         <v>321</v>
       </c>
       <c r="AM19" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AN19" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="AO19">
-        <v>0.99730422320290779</v>
+        <v>0.9963019969989696</v>
       </c>
       <c r="AP19">
-        <v>49.422574613357185</v>
+        <v>67.796721685557472</v>
       </c>
       <c r="AR19" t="s">
         <v>240</v>
@@ -8638,16 +8638,16 @@
         <v>400</v>
       </c>
       <c r="BA19" t="s">
+        <v>419</v>
+      </c>
+      <c r="BB19" t="s">
         <v>420</v>
       </c>
-      <c r="BB19" t="s">
-        <v>417</v>
-      </c>
       <c r="BC19">
-        <v>0.99564789206089888</v>
+        <v>0.99353710926584593</v>
       </c>
       <c r="BD19">
-        <v>79.788645550187297</v>
+        <v>118.48633012615811</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -8712,16 +8712,16 @@
         <v>261</v>
       </c>
       <c r="Y20" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="Z20" t="s">
         <v>294</v>
       </c>
       <c r="AA20">
-        <v>0.99812712894455979</v>
+        <v>0.99801094175818605</v>
       </c>
       <c r="AB20">
-        <v>34.335969349736395</v>
+        <v>36.466067766588218</v>
       </c>
       <c r="AD20" t="s">
         <v>240</v>
@@ -8748,16 +8748,16 @@
         <v>323</v>
       </c>
       <c r="AM20" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="AN20" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AO20">
-        <v>0.99805709209211746</v>
+        <v>0.99635146162488653</v>
       </c>
       <c r="AP20">
-        <v>35.619978311179104</v>
+        <v>66.889870210414614</v>
       </c>
       <c r="AR20" t="s">
         <v>240</v>
@@ -8858,16 +8858,16 @@
         <v>263</v>
       </c>
       <c r="Y21" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="Z21" t="s">
         <v>295</v>
       </c>
       <c r="AA21">
-        <v>0.99834158364926728</v>
+        <v>0.99909366739195871</v>
       </c>
       <c r="AB21">
-        <v>30.404299763434018</v>
+        <v>16.616097814091063</v>
       </c>
       <c r="AD21" t="s">
         <v>240</v>
@@ -8894,16 +8894,16 @@
         <v>325</v>
       </c>
       <c r="AM21" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AN21" t="s">
-        <v>365</v>
+        <v>287</v>
       </c>
       <c r="AO21">
-        <v>0.99641308487583879</v>
+        <v>0.99586212495478665</v>
       </c>
       <c r="AP21">
-        <v>65.760110609622657</v>
+        <v>75.861042495577635</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -8968,16 +8968,16 @@
         <v>265</v>
       </c>
       <c r="Y22" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Z22" t="s">
         <v>296</v>
       </c>
       <c r="AA22">
-        <v>0.9987403722896917</v>
+        <v>0.99839233674974392</v>
       </c>
       <c r="AB22">
-        <v>23.093174688985375</v>
+        <v>29.473826254695162</v>
       </c>
       <c r="AD22" t="s">
         <v>240</v>
@@ -9010,10 +9010,10 @@
         <v>367</v>
       </c>
       <c r="AO22">
-        <v>0.99449756685866841</v>
+        <v>0.99653588726932718</v>
       </c>
       <c r="AP22">
-        <v>100.87794092441324</v>
+        <v>63.508733395668145</v>
       </c>
     </row>
     <row r="23" spans="2:56">
@@ -9078,16 +9078,16 @@
         <v>267</v>
       </c>
       <c r="Y23" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="Z23" t="s">
         <v>297</v>
       </c>
       <c r="AA23">
-        <v>0.99801094175818605</v>
+        <v>0.99729953359766199</v>
       </c>
       <c r="AB23">
-        <v>36.466067766588218</v>
+        <v>49.508550709529651</v>
       </c>
       <c r="AD23" t="s">
         <v>240</v>
@@ -9120,10 +9120,10 @@
         <v>369</v>
       </c>
       <c r="AO23">
-        <v>0.99845079995590791</v>
+        <v>0.99826576737141715</v>
       </c>
       <c r="AP23">
-        <v>28.402000808355538</v>
+        <v>31.794264857351436</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -9188,16 +9188,16 @@
         <v>269</v>
       </c>
       <c r="Y24" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="Z24" t="s">
         <v>298</v>
       </c>
       <c r="AA24">
-        <v>0.99909366739195871</v>
+        <v>0.99812712894455979</v>
       </c>
       <c r="AB24">
-        <v>16.616097814091063</v>
+        <v>34.335969349736395</v>
       </c>
       <c r="AD24" t="s">
         <v>240</v>
@@ -9230,10 +9230,10 @@
         <v>371</v>
       </c>
       <c r="AO24">
-        <v>0.9963019969989696</v>
+        <v>0.99871360797890252</v>
       </c>
       <c r="AP24">
-        <v>67.796721685557472</v>
+        <v>23.583853720120768</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -9298,16 +9298,16 @@
         <v>271</v>
       </c>
       <c r="Y25" t="s">
-        <v>234</v>
+        <v>221</v>
       </c>
       <c r="Z25" t="s">
         <v>299</v>
       </c>
       <c r="AA25">
-        <v>0.99839233674974392</v>
+        <v>0.99834158364926728</v>
       </c>
       <c r="AB25">
-        <v>29.473826254695162</v>
+        <v>30.404299763434018</v>
       </c>
       <c r="AD25" t="s">
         <v>240</v>
@@ -9340,10 +9340,10 @@
         <v>373</v>
       </c>
       <c r="AO25">
-        <v>0.99776911581804295</v>
+        <v>0.99883902037019667</v>
       </c>
       <c r="AP25">
-        <v>40.899543335879912</v>
+        <v>21.284626546395259</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -9408,16 +9408,16 @@
         <v>273</v>
       </c>
       <c r="Y26" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="Z26" t="s">
         <v>300</v>
       </c>
       <c r="AA26">
-        <v>0.99572127940552169</v>
+        <v>0.9987403722896917</v>
       </c>
       <c r="AB26">
-        <v>78.443210898768598</v>
+        <v>23.093174688985375</v>
       </c>
       <c r="AD26" t="s">
         <v>240</v>
@@ -9450,10 +9450,10 @@
         <v>375</v>
       </c>
       <c r="AO26">
-        <v>0.99802303154782224</v>
+        <v>0.99521984547821263</v>
       </c>
       <c r="AP26">
-        <v>36.244421623259619</v>
+        <v>87.636166232768815</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -9518,16 +9518,16 @@
         <v>275</v>
       </c>
       <c r="Y27" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="Z27" t="s">
         <v>301</v>
       </c>
       <c r="AA27">
-        <v>0.99738245649758195</v>
+        <v>0.99763459325217896</v>
       </c>
       <c r="AB27">
-        <v>47.988297544331637</v>
+        <v>43.365790376719588</v>
       </c>
       <c r="AD27" t="s">
         <v>240</v>
@@ -9560,10 +9560,10 @@
         <v>377</v>
       </c>
       <c r="AO27">
-        <v>0.99714358927215652</v>
+        <v>0.99730422320290779</v>
       </c>
       <c r="AP27">
-        <v>52.367530010463909</v>
+        <v>49.422574613357185</v>
       </c>
     </row>
     <row r="28" spans="2:56">
@@ -9628,16 +9628,16 @@
         <v>277</v>
       </c>
       <c r="Y28" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="Z28" t="s">
         <v>302</v>
       </c>
       <c r="AA28">
-        <v>0.99763459325217896</v>
+        <v>0.99505524223378883</v>
       </c>
       <c r="AB28">
-        <v>43.365790376719588</v>
+        <v>90.653892380538664</v>
       </c>
       <c r="AD28" t="s">
         <v>240</v>
@@ -9670,10 +9670,10 @@
         <v>379</v>
       </c>
       <c r="AO28">
-        <v>0.99749126227646956</v>
+        <v>0.99805709209211746</v>
       </c>
       <c r="AP28">
-        <v>45.993524931390482</v>
+        <v>35.619978311179104</v>
       </c>
     </row>
     <row r="29" spans="2:56">
@@ -9738,16 +9738,16 @@
         <v>279</v>
       </c>
       <c r="Y29" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="Z29" t="s">
         <v>303</v>
       </c>
       <c r="AA29">
-        <v>0.99505524223378883</v>
+        <v>0.99860106452186825</v>
       </c>
       <c r="AB29">
-        <v>90.653892380538664</v>
+        <v>25.647150432415483</v>
       </c>
       <c r="AD29" t="s">
         <v>240</v>
@@ -9780,10 +9780,10 @@
         <v>381</v>
       </c>
       <c r="AO29">
-        <v>0.99807543246352515</v>
+        <v>0.99802303154782224</v>
       </c>
       <c r="AP29">
-        <v>35.283738168705199</v>
+        <v>36.244421623259619</v>
       </c>
     </row>
     <row r="30" spans="2:56">
@@ -9848,16 +9848,16 @@
         <v>281</v>
       </c>
       <c r="Y30" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="Z30" t="s">
         <v>304</v>
       </c>
       <c r="AA30">
-        <v>0.99692898913090644</v>
+        <v>0.99775856069920277</v>
       </c>
       <c r="AB30">
-        <v>56.301865933381954</v>
+        <v>41.093053847949164</v>
       </c>
       <c r="AD30" t="s">
         <v>240</v>
@@ -9890,10 +9890,10 @@
         <v>383</v>
       </c>
       <c r="AO30">
-        <v>0.99622969699231045</v>
+        <v>0.99714358927215652</v>
       </c>
       <c r="AP30">
-        <v>69.122221807641537</v>
+        <v>52.367530010463909</v>
       </c>
     </row>
   </sheetData>
@@ -9902,7 +9902,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA04E66F-EC3B-4029-AC28-E3A39D910DC3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2DF36F-B208-4F92-A495-60148317DEFE}">
   <dimension ref="B9:Z30"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -10014,7 +10014,7 @@
         <v>423</v>
       </c>
       <c r="K11" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="L11">
         <v>0.30278350605008381</v>
@@ -10047,7 +10047,7 @@
         <v>463</v>
       </c>
       <c r="X11" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="Y11">
         <v>0.83925000000000005</v>
@@ -10082,7 +10082,7 @@
         <v>425</v>
       </c>
       <c r="K12" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="L12">
         <v>0.44035497786033617</v>
@@ -10115,7 +10115,7 @@
         <v>465</v>
       </c>
       <c r="X12" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="Y12">
         <v>16.887</v>
@@ -10150,7 +10150,7 @@
         <v>427</v>
       </c>
       <c r="K13" t="s">
-        <v>380</v>
+        <v>355</v>
       </c>
       <c r="L13">
         <v>1.6077871713950227</v>
@@ -10183,7 +10183,7 @@
         <v>467</v>
       </c>
       <c r="X13" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="Y13">
         <v>11.2965</v>
@@ -10218,7 +10218,7 @@
         <v>429</v>
       </c>
       <c r="K14" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="L14">
         <v>2.531891424764753</v>
@@ -10251,7 +10251,7 @@
         <v>469</v>
       </c>
       <c r="X14" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="Y14">
         <v>6.6577500000000001</v>
@@ -10286,7 +10286,7 @@
         <v>431</v>
       </c>
       <c r="K15" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="L15">
         <v>7.6497810049421515</v>
@@ -10319,7 +10319,7 @@
         <v>471</v>
       </c>
       <c r="X15" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="Y15">
         <v>17.089500000000001</v>
@@ -10354,7 +10354,7 @@
         <v>433</v>
       </c>
       <c r="K16" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="L16">
         <v>0.63333325583919986</v>
@@ -10387,7 +10387,7 @@
         <v>473</v>
       </c>
       <c r="X16" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="Y16">
         <v>8.8230000000000004</v>
@@ -10422,7 +10422,7 @@
         <v>435</v>
       </c>
       <c r="K17" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="L17">
         <v>0.78389041837100704</v>
@@ -10455,7 +10455,7 @@
         <v>475</v>
       </c>
       <c r="X17" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="Y17">
         <v>0.22650000000000001</v>
@@ -10490,7 +10490,7 @@
         <v>437</v>
       </c>
       <c r="K18" t="s">
-        <v>352</v>
+        <v>374</v>
       </c>
       <c r="L18">
         <v>3.0365724666245324</v>
@@ -10523,7 +10523,7 @@
         <v>477</v>
       </c>
       <c r="X18" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="Y18">
         <v>9.5062499999999996</v>
@@ -10558,7 +10558,7 @@
         <v>439</v>
       </c>
       <c r="K19" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="L19">
         <v>0.22970161230087291</v>
@@ -10626,7 +10626,7 @@
         <v>441</v>
       </c>
       <c r="K20" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="L20">
         <v>0.27066515065379043</v>
@@ -10659,7 +10659,7 @@
         <v>481</v>
       </c>
       <c r="X20" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
       <c r="Y20">
         <v>3.9427500000000002</v>
@@ -10694,7 +10694,7 @@
         <v>443</v>
       </c>
       <c r="K21" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="L21">
         <v>0.32193208719379746</v>
@@ -10729,7 +10729,7 @@
         <v>445</v>
       </c>
       <c r="K22" t="s">
-        <v>378</v>
+        <v>353</v>
       </c>
       <c r="L22">
         <v>0.6573344927201471</v>
@@ -10764,7 +10764,7 @@
         <v>447</v>
       </c>
       <c r="K23" t="s">
-        <v>350</v>
+        <v>372</v>
       </c>
       <c r="L23">
         <v>0.28992997651770519</v>
@@ -10799,7 +10799,7 @@
         <v>449</v>
       </c>
       <c r="K24" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="L24">
         <v>0.74609319967150689</v>
@@ -10834,7 +10834,7 @@
         <v>451</v>
       </c>
       <c r="K25" t="s">
-        <v>364</v>
+        <v>345</v>
       </c>
       <c r="L25">
         <v>0.35328950844501877</v>
@@ -10869,7 +10869,7 @@
         <v>453</v>
       </c>
       <c r="K26" t="s">
-        <v>366</v>
+        <v>347</v>
       </c>
       <c r="L26">
         <v>0.7924639655878376</v>
@@ -10904,7 +10904,7 @@
         <v>455</v>
       </c>
       <c r="K27" t="s">
-        <v>372</v>
+        <v>349</v>
       </c>
       <c r="L27">
         <v>0.55411362221124194</v>
@@ -10939,7 +10939,7 @@
         <v>457</v>
       </c>
       <c r="K28" t="s">
-        <v>382</v>
+        <v>357</v>
       </c>
       <c r="L28">
         <v>1.4327274230737423</v>
@@ -10974,7 +10974,7 @@
         <v>459</v>
       </c>
       <c r="K29" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="L29">
         <v>0.58742801517356968</v>
@@ -11009,7 +11009,7 @@
         <v>461</v>
       </c>
       <c r="K30" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
       <c r="L30">
         <v>0.35405891742987328</v>
@@ -11024,7 +11024,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED0E8BD3-674E-4FD9-B03B-D37DEE656B5F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5FEA79-DBE7-4722-9963-B0FD82681EC1}">
   <dimension ref="B9:S128"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -14526,7 +14526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{904B39ED-F08F-40AD-AC13-E0D210BEA885}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B63E126-0A6F-4058-BD81-7D35D7CB13D5}">
   <dimension ref="B2:M87"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15599,7 +15599,7 @@
         <v>576</v>
       </c>
       <c r="C36" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="D36" t="s">
         <v>577</v>
@@ -15634,7 +15634,7 @@
         <v>577</v>
       </c>
       <c r="D37" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="E37">
         <v>1</v>

</xml_diff>